<commit_message>
Fix faint spectrograms and remove the dropped two_female clip
Spectrograms were rendering almost blank because the color scale only
covered -40 to 0 dB, but real call energy in these field recordings
sits mostly between -70 and -40 dB - over 90% of the signal was being
crushed into a single background color. Widened the range to -70 to 0
dB so actual call structure is visible.

Also removes two_female_wesoke_maybe.wav (already deleted from wavs/)
from the call log, calls.csv, and generated audio/spectrogram files,
and picks up the team bios that were filled in for Megan, Max, and
Reese.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/call_log.xlsx
+++ b/data/call_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
   <si>
     <t>filename</t>
   </si>
@@ -110,12 +110,6 @@
   </si>
   <si>
     <t>WESOMac_sticatto_morse_code_call.wav</t>
-  </si>
-  <si>
-    <t>two_female_wesoke_maybe.wav</t>
-  </si>
-  <si>
-    <t>Two female maybe</t>
   </si>
 </sst>
 </file>
@@ -458,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
@@ -635,14 +629,6 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" t="s">
-        <v>33</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 11 new call recordings, subspecies display, custom section order
Adds 11 new clips (spectrograms + audio) covering Song, Double Trill,
Barking, Begging, and Abnormal Vocalisations. The call dictionary now
groups sections in a fixed order (Song, Double Trill, Barking, Begging,
Food Delivery Call, Whinny, then any other type, with Abnormal
Vocalisations always last) and shows the subspecies (italicized)
alongside context/location/date for each example.

Also:
- Grammar-only copyedit pass across call_log.xlsx descriptions/context
  (typos, missing articles, comma splices, capitalization consistency)
- Fixed two bugs in sync_from_wavs.R: it silently dropped the new
  subspecies column on every sync, and crashed when the date column
  came back as a real Date type instead of text
- Centered/italicized the "Current Team" and "Alumni" headings on the
  About page

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/call_log.xlsx
+++ b/data/call_log.xlsx
@@ -14,11 +14,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="77">
   <si>
     <t>filename</t>
   </si>
   <si>
+    <t>subspecies</t>
+  </si>
+  <si>
     <t>call_type</t>
   </si>
   <si>
@@ -37,13 +40,22 @@
     <t>morse_code_call_wesomac.wav</t>
   </si>
   <si>
-    <t>Food Delivery: Call</t>
+    <t>M. k. macfarlanei</t>
+  </si>
+  <si>
+    <t>Food Delivery Call</t>
+  </si>
+  <si>
+    <t>Male calling while approaching the nest box with food.</t>
   </si>
   <si>
     <t>Kaleden, B.C.</t>
   </si>
   <si>
-    <t>These short, staccato calls are always heard in relation to food being brought to the nest.</t>
+    <t>2022-05-27</t>
+  </si>
+  <si>
+    <t>Food delivery calls are unique and highly context-dependent. They have only ever been observed in relation to prey deliveries to the nest; however, they may also be used as a form of intimate contact call, but this has not been looked at. They often consist of short staccato notes, much like morse code.</t>
   </si>
   <si>
     <t>WESOmac_barking.wav</t>
@@ -52,64 +64,187 @@
     <t>Barking</t>
   </si>
   <si>
-    <t>Barks are loud, short bursts with lots of harmonics, and are usually a sign that an owl is agitated. They're typically heard from the female once the chicks are a little older or have fledged; however, they can occur whenever an owl is agitated, potentially in response to a predator, often a non-volant one (e.g. human, dog, raccoon, etc.).</t>
+    <t>Female barking after leaving the nest.</t>
+  </si>
+  <si>
+    <t>Barks are loud, short bursts with lots of harmonics, and are usually a sign that an owl is agitated. They're typically heard from the female once the chicks are a little older or have fledged; however, they can occur whenever an owl is agitated, often in response to a predator.</t>
   </si>
   <si>
     <t>WESOmac_Chick1.wav</t>
   </si>
   <si>
-    <t>Chick Begging</t>
-  </si>
-  <si>
-    <t>Chicks will often, but not always, beg for food from their parents. This most often happens at the beginning of the evening, before they've been fed, and it tapers off as they become satiated. However, some chicks won't beg as often if the brood size is small, since chicks tend to be more satiated compared to nests with a larger brood, where chicks need to vie for food against their brood-mates.</t>
+    <t>Begging</t>
+  </si>
+  <si>
+    <t>Chicks within the nest box, perhaps 2-3 weeks old.</t>
+  </si>
+  <si>
+    <t>Begging is a form of demand. Often begging is a bid for affection or food. Although males have not been observed begging, they likely can. Both adult female owls and chicks will beg frequently during the breeding season. Chick begging progresses as they grow, and chicks will continue to be distinguishable from adult female begging until 2-3 months after they are fledged. Once owls have matured in the fall, they become unrecognisable from adults.</t>
   </si>
   <si>
     <t>WESOmac_Chick2.wav</t>
   </si>
   <si>
+    <t>Chicks within the nest cavity, perhaps 2-3 weeks old.</t>
+  </si>
+  <si>
+    <t>Okanagan Falls, B.C.</t>
+  </si>
+  <si>
+    <t>2022-05-28</t>
+  </si>
+  <si>
     <t>WESOmac_Chick3.wav</t>
   </si>
   <si>
+    <t>2022-05-26</t>
+  </si>
+  <si>
     <t>WESOmac_Chick4_young.wav</t>
   </si>
   <si>
+    <t>Chicks within the nest box, perhaps 1-2 weeks old.</t>
+  </si>
+  <si>
+    <t>2022-05-17</t>
+  </si>
+  <si>
     <t>WESOmac_doubletrill.wav</t>
   </si>
   <si>
-    <t>Song: Double Trill</t>
-  </si>
-  <si>
-    <t>Males often give a double-trill as a more aggressive song, sometimes heard in response to call playback.</t>
+    <t>Double Trill</t>
+  </si>
+  <si>
+    <t>Male singing near the nest box.</t>
+  </si>
+  <si>
+    <t>Both males and females will give a double-trill as a more aggressive form of their song, sometimes heard in response to call playback.</t>
   </si>
   <si>
     <t>WESOmac_femalebeg.wav</t>
   </si>
   <si>
-    <t>Female: Begging</t>
-  </si>
-  <si>
-    <t>Females, like chicks, will often utter a begging call to males when they are hungry or wanting attention.</t>
+    <t>Adult female owl begging for food from the male. She is in the nest box.</t>
   </si>
   <si>
     <t>WESOmac_femaledrumming.wav</t>
   </si>
   <si>
-    <t>Female: Drumming</t>
-  </si>
-  <si>
-    <t>Females will drum; however, there are very few observations of this behaviour, and it's unclear exactly what the drumming signifies. This is much less understood than drumming in males.</t>
+    <t>Drumming</t>
+  </si>
+  <si>
+    <t>Female in the nest box, similar to male drumming, but the chicks were roughly 2-3 weeks old at this point.</t>
+  </si>
+  <si>
+    <t>Drumming is most often heard from the male prior to copulation. In some contexts, owls have also been heard drumming from within the nest cavity. Drumming does not have a set duration but can continue for several minutes and consists of short, evenly measured notes, often not broadcast loudly. Most often the male will drum when the female is nearby, but drumming has been observed in other contexts as well. The context of female drumming is less clearly understood.</t>
   </si>
   <si>
     <t>WESOmac_femalewhinnying2.wav</t>
   </si>
   <si>
-    <t>Female: Whinny</t>
-  </si>
-  <si>
-    <t>Like the begging call, females will utter a whinny as either a contact call or a bid for attention or food.</t>
+    <t>Whinny</t>
+  </si>
+  <si>
+    <t>Female calling in the nest.</t>
+  </si>
+  <si>
+    <t>Begging is a form of demand. Often begging is a bid for affection or food. Although males have not been observed begging, they likely can, but both adult female owls and chicks will beg frequently during the breeding season. Chick begging progresses as they grow and chicks will continue to be distinguishable from adult female begging until 2-3 months after they are fledged. Once owls have matured in the fall, they become unrecognisable from adults.</t>
   </si>
   <si>
     <t>WESOMac_sticatto_morse_code_call.wav</t>
+  </si>
+  <si>
+    <t>barkingweso_and_ghow_may23_2026.wav</t>
+  </si>
+  <si>
+    <t>Female began barking after a Great-Horned Owl started barking.</t>
+  </si>
+  <si>
+    <t>2022-05-23</t>
+  </si>
+  <si>
+    <t>doubletrillmale_2022May22.wav</t>
+  </si>
+  <si>
+    <t>2022-05-22</t>
+  </si>
+  <si>
+    <t>female_abnormal_wesomac_may20_2022.wav</t>
+  </si>
+  <si>
+    <t>Abnormal Vocalisations</t>
+  </si>
+  <si>
+    <t>While the female is in the nest box, these calls may precede a prey delivery to the nest, or serve as an intimate form of contact call.</t>
+  </si>
+  <si>
+    <t>2022-05-20</t>
+  </si>
+  <si>
+    <t>There are a slew of less frequently heard vocalisations - these are used in extreme situations, or are so intimate between owls that they are very rarely heard by observers. These can include calls associated with pain, bill clacking (often heard as a defense or in situations of heightened aggression), and more intimate contact calls between adult owls or between parents and offspring.</t>
+  </si>
+  <si>
+    <t>fledged_chicks_begging_june17_2022.wav</t>
+  </si>
+  <si>
+    <t>A triplet of fledged chicks begging for food from their parents. They are volant but recently fledged, and are not hypermobile yet.</t>
+  </si>
+  <si>
+    <t>Kelowna, B.C.</t>
+  </si>
+  <si>
+    <t>2022-06-17</t>
+  </si>
+  <si>
+    <t>malesong_may20_2022_wesomac.wav</t>
+  </si>
+  <si>
+    <t>Song</t>
+  </si>
+  <si>
+    <t>Both male and female adult Western Screech-Owls can sing. Males often sing at a lower frequency (550-750 Hz), whereas females sing at a higher frequency (800-900 Hz). Males sing more often than females and sing to defend territory and advertise to females. This is the most common and easily recognised of their calls and can be heard most regularly during the breeding season from February through June, but can often be heard at other times of the year as owls delineate their territorial boundaries. Females will sing less frequently and most commonly as a part of a male/female duet or in territorial defense.</t>
+  </si>
+  <si>
+    <t>march24_2026_wesomac_barking.wav</t>
+  </si>
+  <si>
+    <t>Adult owl barking in response to Great-Horned Owl song.</t>
+  </si>
+  <si>
+    <t>2022-05-24</t>
+  </si>
+  <si>
+    <t>May21_2022_wesomac_chick_and_female_begging.wav</t>
+  </si>
+  <si>
+    <t>Both the adult female and one of the chicks are begging from within the nest box.</t>
+  </si>
+  <si>
+    <t>may192026_wesomac_intimatebarks.wav</t>
+  </si>
+  <si>
+    <t>Female in the nest box with chicks. Often heard intimately between the female and chicks, but likely still indicates a milder form of irritation.</t>
+  </si>
+  <si>
+    <t>owwweeee_chicks_May24_202022_wesomac.wav</t>
+  </si>
+  <si>
+    <t>Fighting between nestlings. These vocalisations have often been heard as a pain response or a 'let go'. Similar vocalisations have been heard from Northern Saw-whet Owls once captured by a predator. This does not indicate predation, but is likely a response to discomfort.</t>
+  </si>
+  <si>
+    <t>wesomac_chick_bill_clacking_May24_2022.wav</t>
+  </si>
+  <si>
+    <t>Chick bill clacking at other nestlings within the nest box. Bill clacking is often heard as a defense or a sign of extreme irritation. Often heard while handling owls.</t>
+  </si>
+  <si>
+    <t>WDRP_20220610_2305.wav</t>
+  </si>
+  <si>
+    <t>Chick singing in response to adult male.</t>
+  </si>
+  <si>
+    <t>2022-06-10</t>
   </si>
 </sst>
 </file>
@@ -452,10 +587,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,159 +609,487 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" t="s">
+        <v>54</v>
+      </c>
+      <c r="G17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G18" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="D19" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" t="s">
-        <v>9</v>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" t="s">
+        <v>69</v>
+      </c>
+      <c r="G20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" t="s">
+        <v>71</v>
+      </c>
+      <c r="G21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" t="s">
+        <v>76</v>
+      </c>
+      <c r="G23" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>